<commit_message>
feat(blog,notification): CRUD blog, notification, push notification with web push, real time notification with webnsocket
</commit_message>
<xml_diff>
--- a/docs/samples/timetable-import-sample.xlsx
+++ b/docs/samples/timetable-import-sample.xlsx
@@ -82,61 +82,61 @@
     <t>1 (Sáng)</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.101</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.101</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.101</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.101</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.101</t>
   </si>
   <si>
     <t>2 (Sáng)</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.101</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.101</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.101</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.101</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.101</t>
   </si>
   <si>
     <t>3 (Sáng)</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.101</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.101</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.101</t>
   </si>
   <si>
@@ -167,220 +167,220 @@
     <t>10A2</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.102</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.102</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.102</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.102</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.102</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.102</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.102</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.102</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.102</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.102</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.102</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.102</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.102</t>
   </si>
   <si>
     <t>10A3</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.103</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.103</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.103</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.103</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.103</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.103</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.103</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.103</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.103</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.103</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.103</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.103</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.103</t>
   </si>
   <si>
     <t>10A4</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.104</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.104</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.104</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.104</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.104</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.104</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.104</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.104</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.104</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.104</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.104</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.104</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.104</t>
   </si>
   <si>
     <t>10A5</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.105</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.105</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.105</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.105</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.105</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.105</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.105</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.105</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.105</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.105</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.105</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.105</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.105</t>
   </si>
   <si>
@@ -390,550 +390,550 @@
     <t>Đã điền từ TKB HK2 năm trước (chỉ mã môn)</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.106</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.106</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.106</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.106</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.106</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.106</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.106</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.106</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.106</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.106</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.106</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.106</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.106</t>
   </si>
   <si>
     <t>11A2</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.107</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.107</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.107</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.107</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.107</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.107</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.107</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.107</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.107</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.107</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.107</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.107</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.107</t>
   </si>
   <si>
     <t>11A3</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.108</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.108</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.108</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.108</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.108</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.108</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.108</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.108</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.108</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.108</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.108</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.108</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.108</t>
   </si>
   <si>
     <t>11A4</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.109</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.109</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.109</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.109</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.109</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.109</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.109</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.109</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.109</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.109</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.109</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.109</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.109</t>
   </si>
   <si>
     <t>11A5</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.110</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.110</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.110</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.110</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.110</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.110</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.110</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.110</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.110</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.110</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.110</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.110</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.110</t>
   </si>
   <si>
     <t>12A1</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.111</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.111</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.111</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.111</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.111</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.111</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.111</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.111</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.111</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.111</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.111</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.111</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.111</t>
   </si>
   <si>
     <t>12A2</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.112</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.112</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.112</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.112</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.112</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.112</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.112</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.112</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.112</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.112</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.112</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.112</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.112</t>
   </si>
   <si>
     <t>12A3</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.113</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.113</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.113</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.113</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.113</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.113</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.113</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.113</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.113</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.113</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.113</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.113</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.113</t>
   </si>
   <si>
     <t>12A4</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.114</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.114</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.114</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.114</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.114</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.114</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.114</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.114</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.114</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.114</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.114</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.114</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.114</t>
   </si>
   <si>
     <t>12A5</t>
   </si>
   <si>
-    <t xml:space="preserve">VAN
+    <t xml:space="preserve">Ngữ văn
 P.115</t>
   </si>
   <si>
-    <t xml:space="preserve">TD
+    <t xml:space="preserve">Giáo dục thể chất
 P.115</t>
   </si>
   <si>
-    <t xml:space="preserve">HOA
+    <t xml:space="preserve">Hóa học
 P.115</t>
   </si>
   <si>
-    <t xml:space="preserve">GKTPL
+    <t xml:space="preserve">Giáo dục kinh tế và pháp luật
 P.115</t>
   </si>
   <si>
-    <t xml:space="preserve">DIA
+    <t xml:space="preserve">Địa lý
 P.115</t>
   </si>
   <si>
-    <t xml:space="preserve">ANH
+    <t xml:space="preserve">Tiếng Anh
 P.115</t>
   </si>
   <si>
-    <t xml:space="preserve">CN
+    <t xml:space="preserve">Công nghệ
 P.115</t>
   </si>
   <si>
-    <t xml:space="preserve">SINH
+    <t xml:space="preserve">Sinh học
 P.115</t>
   </si>
   <si>
-    <t xml:space="preserve">TOAN
+    <t xml:space="preserve">Toán học
 P.115</t>
   </si>
   <si>
-    <t xml:space="preserve">TIN
+    <t xml:space="preserve">Tin học
 P.115</t>
   </si>
   <si>
-    <t xml:space="preserve">LY
+    <t xml:space="preserve">Vật lý
 P.115</t>
   </si>
   <si>
-    <t xml:space="preserve">GDQP
+    <t xml:space="preserve">Giáo dục quốc phòng và an ninh
 P.115</t>
   </si>
   <si>
-    <t xml:space="preserve">SU
+    <t xml:space="preserve">Lịch sử
 P.115</t>
   </si>
   <si>
@@ -964,7 +964,7 @@
     <t xml:space="preserve">  Dòng 2 (tuỳ chọn): phòng học (vd. P.101)</t>
   </si>
   <si>
-    <t xml:space="preserve">  Không cần ghi giáo viên — hệ thống lấy GV từ phân công lớp môn</t>
+    <t xml:space="preserve">  Không cần ghi giáo viên — hệ thống đối chiếu Phân công giảng dạy (ACTIVE) theo lớp HC + môn</t>
   </si>
   <si>
     <t>Quy tắc:</t>
@@ -976,7 +976,7 @@
     <t>- Import vào học kỳ đã chọn trên form</t>
   </si>
   <si>
-    <t>- Lớp môn phải đã tồn tại và đã có phân công GV ACTIVE</t>
+    <t>- Ô có môn nhưng chưa phân công GV → bỏ qua (không báo lỗi)</t>
   </si>
   <si>
     <t>- Không trùng tiết trong cùng lớp môn hoặc lịch GV</t>

</xml_diff>